<commit_message>
reorganized data_prep and PKLs
</commit_message>
<xml_diff>
--- a/scripts/redshift_table.xlsx
+++ b/scripts/redshift_table.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\_RschArchives\RSCH3_upload\kl_mmt\scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{159A1610-6782-4509-8DDF-059F94D2B0F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0998224D-0301-43D2-B19C-DFF9F292DFAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{D0472C34-474C-4FE1-B401-AA8D4EBE0D9B}"/>
+    <workbookView xWindow="14865" yWindow="255" windowWidth="13935" windowHeight="14070" xr2:uid="{D0472C34-474C-4FE1-B401-AA8D4EBE0D9B}"/>
   </bookViews>
   <sheets>
     <sheet name="redshift_table" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="907" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="910" uniqueCount="86">
   <si>
     <t>Set_C</t>
   </si>
@@ -6042,6 +6042,9 @@
         <v>33</v>
       </c>
       <c r="N30" s="6"/>
+      <c r="O30" s="4" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="31" spans="1:15" ht="27" customHeight="1">
       <c r="A31" s="3">
@@ -6445,6 +6448,9 @@
         <v>34</v>
       </c>
       <c r="N41" s="6"/>
+      <c r="O41" s="4" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="42" spans="1:15" ht="27" customHeight="1">
       <c r="A42" s="3">
@@ -7501,7 +7507,7 @@
       </c>
       <c r="N71" s="6"/>
       <c r="O71" s="4" t="s">
-        <v>85</v>
+        <v>33</v>
       </c>
     </row>
     <row r="72" spans="1:15" ht="27" customHeight="1">
@@ -9056,6 +9062,9 @@
         <v>16</v>
       </c>
       <c r="N113" s="6"/>
+      <c r="O113" s="4" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="114" spans="1:15" ht="27" customHeight="1">
       <c r="A114" s="3">

</xml_diff>